<commit_message>
defense and torque paper
Revising figures. Will follow up with slightly better figures.
</commit_message>
<xml_diff>
--- a/Documentation/Reports and Papers/Knee_Torque_Test/Tables/PinnedExtensor_GoF.xlsx
+++ b/Documentation/Reports and Papers/Knee_Torque_Test/Tables/PinnedExtensor_GoF.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ExtPinGof" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,21 +16,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-  </numFmts>
-  <fonts count="3">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -44,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -52,28 +45,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <bottom style="thin">
-        <color rgb="00999999"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,266 +417,247 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="58" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Pinned-knee extensor torque-prediction goodness of fit per test, at the adopted correction terms with the stiffness pair locked to the flexor-identified values. Column definitions as in the flexor table. RMSE and maximum absolute residual (Max.) are in N·m; FVU = fraction of variance unexplained. The extensor terms were fitted over the fitting tests, the l0 = 45.7 cm test was held out, and the fitting mean averages the five fitting tests.</t>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Unopt RMSE (N·m)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unopt FVU</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Unopt Max (N·m)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Opt RMSE (N·m)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Opt FVU</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Opt Max (N·m)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Improved BPA char. alone: RMSE (N·m)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Improved BPA char. alone: FVU</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Improved BPA char. alone: Max. (N·m)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Corrected model: RMSE (N·m)</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Corrected model: FVU</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Corrected model: Max. (N·m)</t>
-        </is>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>43.6 cm (training)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2.437</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.9618</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4.284</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.978</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.1634</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1.818</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>l0 = 40.0 cm (fitting)</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>3.092</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>0.5638</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>4.842</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>1.244</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>0.1303</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>2.196</v>
+          <t>43.2 cm tendon (training)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2.878</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4.7304</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4.817</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.525</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.327</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2.481</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>l0 = 40.0 cm, tendon (fitting)</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>3.622</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>6.3919</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>7.845</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>0.8878</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>1.89</v>
+          <t>45.7 cm (training)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2.178</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1.0586</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4.974</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0535</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.206</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>l0 = 43.6 cm (fitting)</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>2.437</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>0.9618</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>4.284</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>0.978</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>0.1634</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>1.818</v>
+          <t>40.0 cm (validation)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3.092</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.5638</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4.842</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.244</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.1303</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2.196</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>l0 = 43.2 cm, tendon (fitting)</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>2.878</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>4.7304</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>4.817</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>1.525</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>1.327</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>2.481</v>
+          <t>40.0 cm tendon (validation)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3.622</v>
+      </c>
+      <c r="C6" t="n">
+        <v>6.3919</v>
+      </c>
+      <c r="D6" t="n">
+        <v>7.845</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.8878</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1.89</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>l0 = 45.7 cm (validation)</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>2.178</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>1.0586</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>4.974</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>0.0535</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>1.206</v>
+          <t>46.5 cm (validation)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.949</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.3152</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.272</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.699</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.1714</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.559</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>l0 = 46.5 cm (fitting)</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>0.949</v>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>0.3152</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>2.272</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>0.699</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>0.1714</v>
-      </c>
-      <c r="G8" s="3" t="n">
-        <v>1.559</v>
+          <t>Mean (training)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2.498</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2.2503</v>
+      </c>
+      <c r="D8" t="n">
+        <v>4.692</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.5145999999999999</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.835</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Mean (fitting, 5 tests)</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>2.596</v>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>2.5926</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>4.812</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>1.159</v>
-      </c>
-      <c r="F9" s="7" t="n">
-        <v>0.536</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>1.989</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Mean (validation)</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
-        <v>2.178</v>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>1.0586</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>4.974</v>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>0.0535</v>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>1.206</v>
+      <c r="B9" t="n">
+        <v>2.554</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2.4236</v>
+      </c>
+      <c r="D9" t="n">
+        <v>4.986</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1.098</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.3965</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.882</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
torque paper and SNS walker work.
</commit_message>
<xml_diff>
--- a/Documentation/Reports and Papers/Knee_Torque_Test/Tables/PinnedExtensor_GoF.xlsx
+++ b/Documentation/Reports and Papers/Knee_Torque_Test/Tables/PinnedExtensor_GoF.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="38" uniqueCount="28">
   <si>
     <t>Test</t>
   </si>
@@ -64,6 +64,39 @@
   </si>
   <si>
     <t>Corrected model Max (N*m)</t>
+  </si>
+  <si>
+    <t>Group</t>
+  </si>
+  <si>
+    <t>l0_cm</t>
+  </si>
+  <si>
+    <t>lten_mm</t>
+  </si>
+  <si>
+    <t>RowLabel</t>
+  </si>
+  <si>
+    <t>Mean</t>
+  </si>
+  <si>
+    <t>CharAlone_RMSE</t>
+  </si>
+  <si>
+    <t>CharAlone_FVU</t>
+  </si>
+  <si>
+    <t>CharAlone_Max</t>
+  </si>
+  <si>
+    <t>Corrected_RMSE</t>
+  </si>
+  <si>
+    <t>Corrected_FVU</t>
+  </si>
+  <si>
+    <t>Corrected_Max</t>
   </si>
 </sst>
 </file>
@@ -109,199 +142,279 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" customWidth="true"/>
-    <col min="2" max="2" width="35.140625" customWidth="true"/>
-    <col min="3" max="3" width="27.85546875" customWidth="true"/>
-    <col min="4" max="4" width="34" customWidth="true"/>
-    <col min="5" max="5" width="27.28515625" customWidth="true"/>
-    <col min="6" max="6" width="20" customWidth="true"/>
-    <col min="7" max="7" width="26.140625" customWidth="true"/>
+    <col min="1" max="1" width="10.28515625" customWidth="true"/>
+    <col min="2" max="2" width="6.28515625" customWidth="true"/>
+    <col min="3" max="3" width="9.140625" customWidth="true"/>
+    <col min="4" max="4" width="9.7109375" customWidth="true"/>
+    <col min="5" max="5" width="16.28515625" customWidth="true"/>
+    <col min="6" max="6" width="15" customWidth="true"/>
+    <col min="7" max="7" width="15.140625" customWidth="true"/>
+    <col min="8" max="8" width="15.7109375" customWidth="true"/>
+    <col min="9" max="9" width="14.42578125" customWidth="true"/>
+    <col min="10" max="10" width="14.5703125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>16</v>
+        <v>24</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="0"/>
+      <c r="B2" s="0">
+        <v>43.600000000000001</v>
+      </c>
       <c r="C2" s="0"/>
       <c r="D2" s="0"/>
-      <c r="E2" s="0"/>
-      <c r="F2" s="0"/>
-      <c r="G2" s="0"/>
+      <c r="E2" s="0">
+        <v>2.4369999999999998</v>
+      </c>
+      <c r="F2" s="0">
+        <v>0.96179999999999999</v>
+      </c>
+      <c r="G2" s="0">
+        <v>4.2839999999999998</v>
+      </c>
+      <c r="H2" s="0">
+        <v>0.97799999999999998</v>
+      </c>
+      <c r="I2" s="0">
+        <v>0.16339999999999999</v>
+      </c>
+      <c r="J2" s="0">
+        <v>1.8180000000000001</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="0">
-        <v>2.4369999999999998</v>
+        <v>43.200000000000003</v>
       </c>
       <c r="C3" s="0">
-        <v>0.96179999999999999</v>
-      </c>
-      <c r="D3" s="0">
-        <v>4.2839999999999998</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="D3" s="0"/>
       <c r="E3" s="0">
-        <v>0.97799999999999998</v>
+        <v>2.8780000000000001</v>
       </c>
       <c r="F3" s="0">
-        <v>0.16339999999999999</v>
+        <v>4.7304000000000004</v>
       </c>
       <c r="G3" s="0">
-        <v>1.8180000000000001</v>
+        <v>4.8170000000000002</v>
+      </c>
+      <c r="H3" s="0">
+        <v>1.5249999999999999</v>
+      </c>
+      <c r="I3" s="0">
+        <v>1.327</v>
+      </c>
+      <c r="J3" s="0">
+        <v>2.4809999999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B4" s="0">
-        <v>2.8780000000000001</v>
-      </c>
-      <c r="C4" s="0">
-        <v>4.7304000000000004</v>
-      </c>
-      <c r="D4" s="0">
-        <v>4.8170000000000002</v>
-      </c>
+        <v>45.700000000000003</v>
+      </c>
+      <c r="C4" s="0"/>
+      <c r="D4" s="0"/>
       <c r="E4" s="0">
-        <v>1.5249999999999999</v>
+        <v>2.1779999999999999</v>
       </c>
       <c r="F4" s="0">
-        <v>1.327</v>
+        <v>1.0586</v>
       </c>
       <c r="G4" s="0">
-        <v>2.4809999999999999</v>
+        <v>4.9740000000000002</v>
+      </c>
+      <c r="H4" s="0">
+        <v>0.48999999999999999</v>
+      </c>
+      <c r="I4" s="0">
+        <v>0.053499999999999999</v>
+      </c>
+      <c r="J4" s="0">
+        <v>1.206</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="0">
-        <v>2.1779999999999999</v>
-      </c>
-      <c r="C5" s="0">
-        <v>1.0586</v>
-      </c>
-      <c r="D5" s="0">
-        <v>4.9740000000000002</v>
+        <v>1</v>
+      </c>
+      <c r="B5" s="0"/>
+      <c r="C5" s="0"/>
+      <c r="D5" s="0" t="s">
+        <v>21</v>
       </c>
       <c r="E5" s="0">
-        <v>0.48999999999999999</v>
+        <v>2.4980000000000002</v>
       </c>
       <c r="F5" s="0">
-        <v>0.053499999999999999</v>
+        <v>2.2503000000000002</v>
       </c>
       <c r="G5" s="0">
-        <v>1.206</v>
+        <v>4.6920000000000002</v>
+      </c>
+      <c r="H5" s="0">
+        <v>0.997</v>
+      </c>
+      <c r="I5" s="0">
+        <v>0.51459999999999995</v>
+      </c>
+      <c r="J5" s="0">
+        <v>1.835</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" s="0">
-        <v>2.4980000000000002</v>
-      </c>
-      <c r="C6" s="0">
-        <v>2.2503000000000002</v>
-      </c>
-      <c r="D6" s="0">
-        <v>4.6920000000000002</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C6" s="0"/>
+      <c r="D6" s="0"/>
       <c r="E6" s="0">
-        <v>0.997</v>
+        <v>3.0920000000000001</v>
       </c>
       <c r="F6" s="0">
-        <v>0.51459999999999995</v>
+        <v>0.56379999999999997</v>
       </c>
       <c r="G6" s="0">
-        <v>1.835</v>
+        <v>4.8419999999999996</v>
+      </c>
+      <c r="H6" s="0">
+        <v>1.244</v>
+      </c>
+      <c r="I6" s="0">
+        <v>0.1303</v>
+      </c>
+      <c r="J6" s="0">
+        <v>2.1960000000000002</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="0"/>
-      <c r="C7" s="0"/>
+      <c r="B7" s="0">
+        <v>40</v>
+      </c>
+      <c r="C7" s="0">
+        <v>40</v>
+      </c>
       <c r="D7" s="0"/>
-      <c r="E7" s="0"/>
-      <c r="F7" s="0"/>
-      <c r="G7" s="0"/>
+      <c r="E7" s="0">
+        <v>3.6219999999999999</v>
+      </c>
+      <c r="F7" s="0">
+        <v>6.3918999999999997</v>
+      </c>
+      <c r="G7" s="0">
+        <v>7.8449999999999998</v>
+      </c>
+      <c r="H7" s="0">
+        <v>1.3500000000000001</v>
+      </c>
+      <c r="I7" s="0">
+        <v>0.88780000000000003</v>
+      </c>
+      <c r="J7" s="0">
+        <v>1.8899999999999999</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="0">
-        <v>3.0920000000000001</v>
-      </c>
-      <c r="C8" s="0">
-        <v>0.56379999999999997</v>
-      </c>
-      <c r="D8" s="0">
-        <v>4.8419999999999996</v>
-      </c>
+        <v>46.5</v>
+      </c>
+      <c r="C8" s="0"/>
+      <c r="D8" s="0"/>
       <c r="E8" s="0">
-        <v>1.244</v>
+        <v>0.94899999999999996</v>
       </c>
       <c r="F8" s="0">
-        <v>0.1303</v>
+        <v>0.31519999999999998</v>
       </c>
       <c r="G8" s="0">
-        <v>2.1960000000000002</v>
+        <v>2.2719999999999998</v>
+      </c>
+      <c r="H8" s="0">
+        <v>0.69899999999999996</v>
+      </c>
+      <c r="I8" s="0">
+        <v>0.1714</v>
+      </c>
+      <c r="J8" s="0">
+        <v>1.559</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="0">
-        <v>3.6219999999999999</v>
-      </c>
-      <c r="C9" s="0">
-        <v>6.3918999999999997</v>
-      </c>
-      <c r="D9" s="0">
-        <v>7.8449999999999998</v>
+        <v>6</v>
+      </c>
+      <c r="B9" s="0"/>
+      <c r="C9" s="0"/>
+      <c r="D9" s="0" t="s">
+        <v>21</v>
       </c>
       <c r="E9" s="0">
-        <v>1.3500000000000001</v>
+        <v>2.5539999999999998</v>
       </c>
       <c r="F9" s="0">
-        <v>0.88780000000000003</v>
+        <v>2.4236</v>
       </c>
       <c r="G9" s="0">
-        <v>1.8899999999999999</v>
+        <v>4.9859999999999998</v>
+      </c>
+      <c r="H9" s="0">
+        <v>1.0980000000000001</v>
+      </c>
+      <c r="I9" s="0">
+        <v>0.39650000000000002</v>
+      </c>
+      <c r="J9" s="0">
+        <v>1.8819999999999999</v>
       </c>
     </row>
     <row r="10">

</xml_diff>